<commit_message>
Add publish-post skill and Publish Status / Publish Date columns to tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KgMES5Qh55NxGa61GMJ3FY
</commit_message>
<xml_diff>
--- a/FB content tracker.xlsx
+++ b/FB content tracker.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:J6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -428,6 +428,8 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -471,6 +473,16 @@
           <t>Post Status</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Publish Status</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Publish Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -513,6 +525,11 @@
           <t>PENDING</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -555,6 +572,11 @@
           <t>PENDING</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -597,6 +619,11 @@
           <t>PENDING</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -639,6 +666,11 @@
           <t>PENDING</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -677,6 +709,11 @@
         </is>
       </c>
       <c r="H6" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>PENDING</t>
         </is>

</xml_diff>